<commit_message>
Add Example Article Versions to 5.1 Sample IR_A1 Report
</commit_message>
<xml_diff>
--- a/source/_static/report/IRA1_sample_r51.xlsx
+++ b/source/_static/report/IRA1_sample_r51.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590DF707-EBB8-42D2-8F7C-A7E2F807AE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B276815-1F4C-44BB-83DF-EB1B46BD5F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="89">
   <si>
     <t>Report_Name</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>P1:1234; ISNI:1234123412341234</t>
+  </si>
+  <si>
+    <t>VoR</t>
   </si>
 </sst>
 </file>
@@ -871,6 +874,9 @@
       <c r="F18" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="G18" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H18" s="1" t="s">
         <v>72</v>
       </c>
@@ -960,6 +966,9 @@
       <c r="F19" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="G19" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H19" s="1" t="s">
         <v>72</v>
       </c>
@@ -1049,6 +1058,9 @@
       <c r="F20" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="G20" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H20" s="1" t="s">
         <v>84</v>
       </c>
@@ -1137,6 +1149,9 @@
       </c>
       <c r="F21" s="1" t="s">
         <v>83</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
Add Article_Versions example to sample IR and IR_A1 (#358)
</commit_message>
<xml_diff>
--- a/source/_static/report/IRA1_sample_r51.xlsx
+++ b/source/_static/report/IRA1_sample_r51.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590DF707-EBB8-42D2-8F7C-A7E2F807AE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B276815-1F4C-44BB-83DF-EB1B46BD5F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="89">
   <si>
     <t>Report_Name</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>P1:1234; ISNI:1234123412341234</t>
+  </si>
+  <si>
+    <t>VoR</t>
   </si>
 </sst>
 </file>
@@ -871,6 +874,9 @@
       <c r="F18" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="G18" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H18" s="1" t="s">
         <v>72</v>
       </c>
@@ -960,6 +966,9 @@
       <c r="F19" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="G19" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H19" s="1" t="s">
         <v>72</v>
       </c>
@@ -1049,6 +1058,9 @@
       <c r="F20" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="G20" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="H20" s="1" t="s">
         <v>84</v>
       </c>
@@ -1137,6 +1149,9 @@
       </c>
       <c r="F21" s="1" t="s">
         <v>83</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>84</v>

</xml_diff>